<commit_message>
Add hotel-detail rate scraper with T1-T4 classification and Excel output
- scraper.py: new scrape_hotel_rates() fetches individual Rakuten hotel pages
  for specified check-in dates (W1/W2/W3 weeks) and classifies room plans
  into T1-T4 types via keyword matching; legacy area-search mode preserved
- cli.py: default mode is now hotel-detail rate collection across the 20 Onnason
  competitor hotels hardcoded from the Excel competitive set; --area-search flag
  retains legacy behaviour; --excel-output fills the 03_料金採取テンプレ sheet
- excel_writer.py: fills the Excel template with scraped rates per hotel/week/type
- __main__.py: allows running as `python -m scraper`
- requirements.txt: add openpyxl>=3.1
- Add Excel template to repo

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013AGLj6WXt47xVsawXoFwja
</commit_message>
<xml_diff>
--- a/沖縄県恩納村エリア_競合料金調査_再構築フレームワーク.xlsx
+++ b/沖縄県恩納村エリア_競合料金調査_再構築フレームワーク.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0\%"/>
   </numFmts>
-  <fonts count="43">
+  <fonts count="45">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -329,6 +329,13 @@
       <b val="1"/>
       <color rgb="FF1F3A5F"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="11">
@@ -460,7 +467,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -811,6 +818,8 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -881,6 +890,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="O4" authorId="0" shapeId="0">
+      <text>
+        <t>2026年7月6日時点でWeb検索により確認したURL（施設名検索結果の上位ページ）。リンク切れ・施設名変更の可能性があるため、Claude in Chrome等でアクセス時に再確認してください。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2210,7 +2234,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="15" customHeight="1" s="59">
       <c r="B25" s="85" t="inlineStr">
         <is>
@@ -2235,12 +2258,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="58" min="1" max="1"/>
     <col width="30" customWidth="1" style="58" min="2" max="2"/>
     <col width="12" customWidth="1" style="58" min="3" max="14"/>
+    <col width="55" customWidth="1" style="59" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.15" customHeight="1" s="59">
@@ -2292,6 +2316,11 @@
       <c r="L4" s="90" t="n"/>
       <c r="M4" s="90" t="n"/>
       <c r="N4" s="90" t="n"/>
+      <c r="O4" s="118" t="inlineStr">
+        <is>
+          <t>楽天トラベルURL</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="59">
       <c r="C5" s="93" t="inlineStr">
@@ -2407,6 +2436,11 @@
       <c r="L7" s="98" t="n"/>
       <c r="M7" s="98" t="n"/>
       <c r="N7" s="98" t="n"/>
+      <c r="O7" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/172611/172611.html</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="59">
       <c r="A8" s="96" t="n">
@@ -2429,6 +2463,11 @@
       <c r="L8" s="98" t="n"/>
       <c r="M8" s="98" t="n"/>
       <c r="N8" s="98" t="n"/>
+      <c r="O8" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/166320/166320.html</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1" s="59">
       <c r="A9" s="96" t="n">
@@ -2451,6 +2490,11 @@
       <c r="L9" s="98" t="n"/>
       <c r="M9" s="98" t="n"/>
       <c r="N9" s="98" t="n"/>
+      <c r="O9" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/16123/16123.html</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1" s="59">
       <c r="A10" s="96" t="n">
@@ -2473,6 +2517,11 @@
       <c r="L10" s="98" t="n"/>
       <c r="M10" s="98" t="n"/>
       <c r="N10" s="98" t="n"/>
+      <c r="O10" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/13554/13554.html</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="59">
       <c r="A11" s="96" t="n">
@@ -2495,6 +2544,11 @@
       <c r="L11" s="98" t="n"/>
       <c r="M11" s="98" t="n"/>
       <c r="N11" s="98" t="n"/>
+      <c r="O11" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/54315/54315.html</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="59">
       <c r="A12" s="96" t="n">
@@ -2517,6 +2571,11 @@
       <c r="L12" s="98" t="n"/>
       <c r="M12" s="98" t="n"/>
       <c r="N12" s="98" t="n"/>
+      <c r="O12" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/141596/141596.html</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1" s="59">
       <c r="A13" s="96" t="n">
@@ -2539,6 +2598,11 @@
       <c r="L13" s="98" t="n"/>
       <c r="M13" s="98" t="n"/>
       <c r="N13" s="98" t="n"/>
+      <c r="O13" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/14275/14275.html</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1" s="59">
       <c r="A14" s="96" t="n">
@@ -2561,6 +2625,11 @@
       <c r="L14" s="98" t="n"/>
       <c r="M14" s="98" t="n"/>
       <c r="N14" s="98" t="n"/>
+      <c r="O14" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/52229/52229.html</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1" s="59">
       <c r="A15" s="96" t="n">
@@ -2583,6 +2652,11 @@
       <c r="L15" s="98" t="n"/>
       <c r="M15" s="98" t="n"/>
       <c r="N15" s="98" t="n"/>
+      <c r="O15" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/15483/15483.html</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1" s="59">
       <c r="A16" s="96" t="n">
@@ -2605,6 +2679,11 @@
       <c r="L16" s="98" t="n"/>
       <c r="M16" s="98" t="n"/>
       <c r="N16" s="98" t="n"/>
+      <c r="O16" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/78239/78239.html</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1" s="59">
       <c r="A17" s="96" t="n">
@@ -2627,6 +2706,11 @@
       <c r="L17" s="98" t="n"/>
       <c r="M17" s="98" t="n"/>
       <c r="N17" s="98" t="n"/>
+      <c r="O17" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/70318/70318.html</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1" s="59">
       <c r="A18" s="96" t="n">
@@ -2649,6 +2733,11 @@
       <c r="L18" s="98" t="n"/>
       <c r="M18" s="98" t="n"/>
       <c r="N18" s="98" t="n"/>
+      <c r="O18" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/180687/180687.html</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1" s="59">
       <c r="A19" s="96" t="n">
@@ -2671,6 +2760,11 @@
       <c r="L19" s="98" t="n"/>
       <c r="M19" s="98" t="n"/>
       <c r="N19" s="98" t="n"/>
+      <c r="O19" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/183576/183576.html</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1" s="59">
       <c r="A20" s="96" t="n">
@@ -2693,6 +2787,11 @@
       <c r="L20" s="98" t="n"/>
       <c r="M20" s="98" t="n"/>
       <c r="N20" s="98" t="n"/>
+      <c r="O20" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/179815/179815.html</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1" s="59">
       <c r="A21" s="96" t="n">
@@ -2715,6 +2814,11 @@
       <c r="L21" s="98" t="n"/>
       <c r="M21" s="98" t="n"/>
       <c r="N21" s="98" t="n"/>
+      <c r="O21" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/104679/104679.html</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1" s="59">
       <c r="A22" s="96" t="n">
@@ -2737,6 +2841,11 @@
       <c r="L22" s="98" t="n"/>
       <c r="M22" s="98" t="n"/>
       <c r="N22" s="98" t="n"/>
+      <c r="O22" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/184015/184015.html</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="59">
       <c r="A23" s="96" t="n">
@@ -2759,6 +2868,11 @@
       <c r="L23" s="98" t="n"/>
       <c r="M23" s="98" t="n"/>
       <c r="N23" s="98" t="n"/>
+      <c r="O23" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/158440/158440.html</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="59">
       <c r="A24" s="96" t="n">
@@ -2781,6 +2895,11 @@
       <c r="L24" s="98" t="n"/>
       <c r="M24" s="98" t="n"/>
       <c r="N24" s="98" t="n"/>
+      <c r="O24" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/164539/164539.html</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1" s="59">
       <c r="A25" s="96" t="n">
@@ -2803,6 +2922,11 @@
       <c r="L25" s="98" t="n"/>
       <c r="M25" s="98" t="n"/>
       <c r="N25" s="98" t="n"/>
+      <c r="O25" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/107650/107650.html</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="59">
       <c r="A26" s="96" t="n">
@@ -2825,6 +2949,11 @@
       <c r="L26" s="98" t="n"/>
       <c r="M26" s="98" t="n"/>
       <c r="N26" s="98" t="n"/>
+      <c r="O26" s="119" t="inlineStr">
+        <is>
+          <t>https://travel.rakuten.co.jp/HOTEL/76791/76791.html</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="59">
       <c r="B28" s="102" t="inlineStr">
@@ -2949,9 +3078,32 @@
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId20"/>
+  </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>